<commit_message>
subo cambios y mediciones
</commit_message>
<xml_diff>
--- a/results/22-02-24/permitividades.xlsx
+++ b/results/22-02-24/permitividades.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AGUA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ACETONA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ISOPR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="agua" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="acetona" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9303,4446 +9302,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C402"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Frecuencia (Hz)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Er Real</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Er Imag</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>100000000</v>
-      </c>
-      <c r="B2" t="n">
-        <v>35.9452608893446</v>
-      </c>
-      <c r="C2" t="n">
-        <v>-4.39770654708642</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>124750000</v>
-      </c>
-      <c r="B3" t="n">
-        <v>38.92817583552245</v>
-      </c>
-      <c r="C3" t="n">
-        <v>-6.424541393347455</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>149500000</v>
-      </c>
-      <c r="B4" t="n">
-        <v>38.16242671946685</v>
-      </c>
-      <c r="C4" t="n">
-        <v>-8.519138772660876</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>174250000</v>
-      </c>
-      <c r="B5" t="n">
-        <v>36.97507597104481</v>
-      </c>
-      <c r="C5" t="n">
-        <v>-9.10988980479906</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>199000000</v>
-      </c>
-      <c r="B6" t="n">
-        <v>35.5213406882076</v>
-      </c>
-      <c r="C6" t="n">
-        <v>-9.990377357171461</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>223750000</v>
-      </c>
-      <c r="B7" t="n">
-        <v>35.61422962256848</v>
-      </c>
-      <c r="C7" t="n">
-        <v>-10.80752849674546</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>248500000</v>
-      </c>
-      <c r="B8" t="n">
-        <v>34.67946372023726</v>
-      </c>
-      <c r="C8" t="n">
-        <v>-11.61212878023326</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>273249984</v>
-      </c>
-      <c r="B9" t="n">
-        <v>33.01237466322372</v>
-      </c>
-      <c r="C9" t="n">
-        <v>-11.91203444509854</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>298000000</v>
-      </c>
-      <c r="B10" t="n">
-        <v>33.31466416318058</v>
-      </c>
-      <c r="C10" t="n">
-        <v>-12.86477858585805</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>322750016</v>
-      </c>
-      <c r="B11" t="n">
-        <v>31.52336895481766</v>
-      </c>
-      <c r="C11" t="n">
-        <v>-13.54540886335716</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>347500000</v>
-      </c>
-      <c r="B12" t="n">
-        <v>30.23377587684961</v>
-      </c>
-      <c r="C12" t="n">
-        <v>-13.91034531659264</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>372249984</v>
-      </c>
-      <c r="B13" t="n">
-        <v>30.05949889302381</v>
-      </c>
-      <c r="C13" t="n">
-        <v>-14.75195196853697</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>397000000</v>
-      </c>
-      <c r="B14" t="n">
-        <v>29.38036334482766</v>
-      </c>
-      <c r="C14" t="n">
-        <v>-15.04646424020819</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>421750016</v>
-      </c>
-      <c r="B15" t="n">
-        <v>27.65975155677947</v>
-      </c>
-      <c r="C15" t="n">
-        <v>-14.91033904359621</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>446500000</v>
-      </c>
-      <c r="B16" t="n">
-        <v>26.27819533767435</v>
-      </c>
-      <c r="C16" t="n">
-        <v>-15.01660790660665</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>471249984</v>
-      </c>
-      <c r="B17" t="n">
-        <v>26.09944740199801</v>
-      </c>
-      <c r="C17" t="n">
-        <v>-14.80429508047898</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>496000000</v>
-      </c>
-      <c r="B18" t="n">
-        <v>26.05881335551401</v>
-      </c>
-      <c r="C18" t="n">
-        <v>-14.62855829753256</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>520750016</v>
-      </c>
-      <c r="B19" t="n">
-        <v>25.23292828443707</v>
-      </c>
-      <c r="C19" t="n">
-        <v>-15.1148503995331</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>545500032</v>
-      </c>
-      <c r="B20" t="n">
-        <v>23.95320402986635</v>
-      </c>
-      <c r="C20" t="n">
-        <v>-15.26698832035004</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>570249984</v>
-      </c>
-      <c r="B21" t="n">
-        <v>23.13579723123557</v>
-      </c>
-      <c r="C21" t="n">
-        <v>-14.88185471779643</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>595000000</v>
-      </c>
-      <c r="B22" t="n">
-        <v>22.81016103037994</v>
-      </c>
-      <c r="C22" t="n">
-        <v>-15.37301470838046</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>619750016</v>
-      </c>
-      <c r="B23" t="n">
-        <v>22.18900821842491</v>
-      </c>
-      <c r="C23" t="n">
-        <v>-15.27214715027489</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>644499968</v>
-      </c>
-      <c r="B24" t="n">
-        <v>21.33344902530457</v>
-      </c>
-      <c r="C24" t="n">
-        <v>-14.69721459815486</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>669249984</v>
-      </c>
-      <c r="B25" t="n">
-        <v>20.92786043621346</v>
-      </c>
-      <c r="C25" t="n">
-        <v>-14.89496116421241</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>694000000</v>
-      </c>
-      <c r="B26" t="n">
-        <v>20.17579256211833</v>
-      </c>
-      <c r="C26" t="n">
-        <v>-14.48100502842682</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>718750016</v>
-      </c>
-      <c r="B27" t="n">
-        <v>20.06792140514187</v>
-      </c>
-      <c r="C27" t="n">
-        <v>-14.50389619159274</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>743500032</v>
-      </c>
-      <c r="B28" t="n">
-        <v>19.68438136967082</v>
-      </c>
-      <c r="C28" t="n">
-        <v>-13.92389184507328</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>768249984</v>
-      </c>
-      <c r="B29" t="n">
-        <v>18.81325618380802</v>
-      </c>
-      <c r="C29" t="n">
-        <v>-13.80253349052616</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>793000000</v>
-      </c>
-      <c r="B30" t="n">
-        <v>18.46651851388348</v>
-      </c>
-      <c r="C30" t="n">
-        <v>-13.73075256705617</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>817750016</v>
-      </c>
-      <c r="B31" t="n">
-        <v>18.29025042013049</v>
-      </c>
-      <c r="C31" t="n">
-        <v>-13.98607636192165</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>842499968</v>
-      </c>
-      <c r="B32" t="n">
-        <v>17.58106523917809</v>
-      </c>
-      <c r="C32" t="n">
-        <v>-14.22039528022144</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>867249984</v>
-      </c>
-      <c r="B33" t="n">
-        <v>17.31044812914915</v>
-      </c>
-      <c r="C33" t="n">
-        <v>-13.5449131668897</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>892000000</v>
-      </c>
-      <c r="B34" t="n">
-        <v>17.13624361707685</v>
-      </c>
-      <c r="C34" t="n">
-        <v>-13.47263040501253</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>916750016</v>
-      </c>
-      <c r="B35" t="n">
-        <v>16.32731817049642</v>
-      </c>
-      <c r="C35" t="n">
-        <v>-12.57758107229641</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>941500032</v>
-      </c>
-      <c r="B36" t="n">
-        <v>16.27755182417801</v>
-      </c>
-      <c r="C36" t="n">
-        <v>-13.42146152735932</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>966249984</v>
-      </c>
-      <c r="B37" t="n">
-        <v>16.00824329863354</v>
-      </c>
-      <c r="C37" t="n">
-        <v>-12.72721562485391</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>991000000</v>
-      </c>
-      <c r="B38" t="n">
-        <v>16.25777168947194</v>
-      </c>
-      <c r="C38" t="n">
-        <v>-12.65781947798775</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>1015750016</v>
-      </c>
-      <c r="B39" t="n">
-        <v>15.56910530038121</v>
-      </c>
-      <c r="C39" t="n">
-        <v>-12.33029857900302</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>1040499968</v>
-      </c>
-      <c r="B40" t="n">
-        <v>15.67098252804787</v>
-      </c>
-      <c r="C40" t="n">
-        <v>-11.95699904594944</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>1065249984</v>
-      </c>
-      <c r="B41" t="n">
-        <v>15.13970100906515</v>
-      </c>
-      <c r="C41" t="n">
-        <v>-11.73929888851667</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>1090000000</v>
-      </c>
-      <c r="B42" t="n">
-        <v>14.71620026561261</v>
-      </c>
-      <c r="C42" t="n">
-        <v>-11.7793982828193</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>1114749952</v>
-      </c>
-      <c r="B43" t="n">
-        <v>15.02798104526003</v>
-      </c>
-      <c r="C43" t="n">
-        <v>-11.77568137736147</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>1139500032</v>
-      </c>
-      <c r="B44" t="n">
-        <v>14.34812230116271</v>
-      </c>
-      <c r="C44" t="n">
-        <v>-11.42196439444914</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>1164249984</v>
-      </c>
-      <c r="B45" t="n">
-        <v>14.30177276760451</v>
-      </c>
-      <c r="C45" t="n">
-        <v>-11.34492463061166</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>1188999936</v>
-      </c>
-      <c r="B46" t="n">
-        <v>14.06943584701094</v>
-      </c>
-      <c r="C46" t="n">
-        <v>-11.16802606983773</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>1213750016</v>
-      </c>
-      <c r="B47" t="n">
-        <v>13.96528621952423</v>
-      </c>
-      <c r="C47" t="n">
-        <v>-10.99854000242018</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>1238499968</v>
-      </c>
-      <c r="B48" t="n">
-        <v>13.7871813286244</v>
-      </c>
-      <c r="C48" t="n">
-        <v>-10.67061353715101</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>1263250048</v>
-      </c>
-      <c r="B49" t="n">
-        <v>13.35489660427191</v>
-      </c>
-      <c r="C49" t="n">
-        <v>-10.59978175256967</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>1288000000</v>
-      </c>
-      <c r="B50" t="n">
-        <v>13.41263846219811</v>
-      </c>
-      <c r="C50" t="n">
-        <v>-10.08427536358195</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>1312749952</v>
-      </c>
-      <c r="B51" t="n">
-        <v>13.11200917852914</v>
-      </c>
-      <c r="C51" t="n">
-        <v>-10.29564166629165</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>1337500032</v>
-      </c>
-      <c r="B52" t="n">
-        <v>12.96389223866674</v>
-      </c>
-      <c r="C52" t="n">
-        <v>-9.988323531999161</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>1362249984</v>
-      </c>
-      <c r="B53" t="n">
-        <v>12.97039578994673</v>
-      </c>
-      <c r="C53" t="n">
-        <v>-9.878919383209514</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>1387000064</v>
-      </c>
-      <c r="B54" t="n">
-        <v>12.6620457275969</v>
-      </c>
-      <c r="C54" t="n">
-        <v>-9.93249107109685</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>1411750016</v>
-      </c>
-      <c r="B55" t="n">
-        <v>12.65879878584574</v>
-      </c>
-      <c r="C55" t="n">
-        <v>-9.894213785121282</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>1436499968</v>
-      </c>
-      <c r="B56" t="n">
-        <v>12.64310390222607</v>
-      </c>
-      <c r="C56" t="n">
-        <v>-9.50330624975118</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>1461250048</v>
-      </c>
-      <c r="B57" t="n">
-        <v>12.30428263492663</v>
-      </c>
-      <c r="C57" t="n">
-        <v>-9.611598474459452</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>1486000000</v>
-      </c>
-      <c r="B58" t="n">
-        <v>12.58588958733186</v>
-      </c>
-      <c r="C58" t="n">
-        <v>-9.209526146750035</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>1510749952</v>
-      </c>
-      <c r="B59" t="n">
-        <v>12.11290909994668</v>
-      </c>
-      <c r="C59" t="n">
-        <v>-9.182436094840822</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>1535500032</v>
-      </c>
-      <c r="B60" t="n">
-        <v>11.92347201350758</v>
-      </c>
-      <c r="C60" t="n">
-        <v>-9.126872591823622</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>1560249984</v>
-      </c>
-      <c r="B61" t="n">
-        <v>11.79822607972716</v>
-      </c>
-      <c r="C61" t="n">
-        <v>-9.000060627364524</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>1584999936</v>
-      </c>
-      <c r="B62" t="n">
-        <v>11.84620031063809</v>
-      </c>
-      <c r="C62" t="n">
-        <v>-8.997405224461033</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>1609750016</v>
-      </c>
-      <c r="B63" t="n">
-        <v>11.95262389242341</v>
-      </c>
-      <c r="C63" t="n">
-        <v>-8.605648228055886</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>1634499968</v>
-      </c>
-      <c r="B64" t="n">
-        <v>11.73924678738291</v>
-      </c>
-      <c r="C64" t="n">
-        <v>-8.46490900330358</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>1659250048</v>
-      </c>
-      <c r="B65" t="n">
-        <v>11.5713848728858</v>
-      </c>
-      <c r="C65" t="n">
-        <v>-8.362380970681299</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>1684000000</v>
-      </c>
-      <c r="B66" t="n">
-        <v>11.56649752053515</v>
-      </c>
-      <c r="C66" t="n">
-        <v>-8.164475975606438</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>1708749952</v>
-      </c>
-      <c r="B67" t="n">
-        <v>11.42403176546924</v>
-      </c>
-      <c r="C67" t="n">
-        <v>-8.110026420537034</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>1733500032</v>
-      </c>
-      <c r="B68" t="n">
-        <v>11.35435354319604</v>
-      </c>
-      <c r="C68" t="n">
-        <v>-8.111466139417409</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>1758249984</v>
-      </c>
-      <c r="B69" t="n">
-        <v>11.31805090469666</v>
-      </c>
-      <c r="C69" t="n">
-        <v>-7.829428860717777</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>1783000064</v>
-      </c>
-      <c r="B70" t="n">
-        <v>11.16832162212556</v>
-      </c>
-      <c r="C70" t="n">
-        <v>-7.693205254637825</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n">
-        <v>1807750016</v>
-      </c>
-      <c r="B71" t="n">
-        <v>11.37987338124793</v>
-      </c>
-      <c r="C71" t="n">
-        <v>-7.816250339915837</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>1832499968</v>
-      </c>
-      <c r="B72" t="n">
-        <v>11.19383657712648</v>
-      </c>
-      <c r="C72" t="n">
-        <v>-7.626736961835066</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="n">
-        <v>1857250048</v>
-      </c>
-      <c r="B73" t="n">
-        <v>11.18629887514354</v>
-      </c>
-      <c r="C73" t="n">
-        <v>-7.673972516527431</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="n">
-        <v>1882000000</v>
-      </c>
-      <c r="B74" t="n">
-        <v>11.02589664606445</v>
-      </c>
-      <c r="C74" t="n">
-        <v>-7.456508096208866</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="n">
-        <v>1906749952</v>
-      </c>
-      <c r="B75" t="n">
-        <v>10.98256493317983</v>
-      </c>
-      <c r="C75" t="n">
-        <v>-7.358314164441699</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>1931500032</v>
-      </c>
-      <c r="B76" t="n">
-        <v>10.94577239865934</v>
-      </c>
-      <c r="C76" t="n">
-        <v>-7.246285582256013</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>1956249984</v>
-      </c>
-      <c r="B77" t="n">
-        <v>10.68743322215767</v>
-      </c>
-      <c r="C77" t="n">
-        <v>-7.174220738701988</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>1980999936</v>
-      </c>
-      <c r="B78" t="n">
-        <v>10.92932667215123</v>
-      </c>
-      <c r="C78" t="n">
-        <v>-7.045233136264176</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>2005750016</v>
-      </c>
-      <c r="B79" t="n">
-        <v>10.75703149277117</v>
-      </c>
-      <c r="C79" t="n">
-        <v>-6.895947548424129</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>2030499968</v>
-      </c>
-      <c r="B80" t="n">
-        <v>10.8516019649282</v>
-      </c>
-      <c r="C80" t="n">
-        <v>-6.976684086998787</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>2055250048</v>
-      </c>
-      <c r="B81" t="n">
-        <v>10.70221826031898</v>
-      </c>
-      <c r="C81" t="n">
-        <v>-6.738950219329628</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>2080000000</v>
-      </c>
-      <c r="B82" t="n">
-        <v>10.79996486816962</v>
-      </c>
-      <c r="C82" t="n">
-        <v>-6.743424259111941</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>2104749952</v>
-      </c>
-      <c r="B83" t="n">
-        <v>10.80381565199886</v>
-      </c>
-      <c r="C83" t="n">
-        <v>-6.568387846263279</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>2129500032</v>
-      </c>
-      <c r="B84" t="n">
-        <v>10.43420042537632</v>
-      </c>
-      <c r="C84" t="n">
-        <v>-6.557571531275213</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>2154249984</v>
-      </c>
-      <c r="B85" t="n">
-        <v>10.37706839774881</v>
-      </c>
-      <c r="C85" t="n">
-        <v>-6.390692972124265</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="n">
-        <v>2179000064</v>
-      </c>
-      <c r="B86" t="n">
-        <v>10.69815302168494</v>
-      </c>
-      <c r="C86" t="n">
-        <v>-6.156131514289692</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n">
-        <v>2203749888</v>
-      </c>
-      <c r="B87" t="n">
-        <v>10.69602023612941</v>
-      </c>
-      <c r="C87" t="n">
-        <v>-6.016341125912173</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="n">
-        <v>2228499968</v>
-      </c>
-      <c r="B88" t="n">
-        <v>10.40914674877068</v>
-      </c>
-      <c r="C88" t="n">
-        <v>-6.152278280397593</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="n">
-        <v>2253250048</v>
-      </c>
-      <c r="B89" t="n">
-        <v>10.12437179234859</v>
-      </c>
-      <c r="C89" t="n">
-        <v>-5.98473951731081</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="n">
-        <v>2278000128</v>
-      </c>
-      <c r="B90" t="n">
-        <v>10.51909065318565</v>
-      </c>
-      <c r="C90" t="n">
-        <v>-6.039987405270812</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>2302749952</v>
-      </c>
-      <c r="B91" t="n">
-        <v>10.41174316781836</v>
-      </c>
-      <c r="C91" t="n">
-        <v>-5.646112440220081</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>2327500032</v>
-      </c>
-      <c r="B92" t="n">
-        <v>10.06457901026573</v>
-      </c>
-      <c r="C92" t="n">
-        <v>-5.750999741172611</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>2352250112</v>
-      </c>
-      <c r="B93" t="n">
-        <v>9.954645112265625</v>
-      </c>
-      <c r="C93" t="n">
-        <v>-5.765936387955302</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>2376999936</v>
-      </c>
-      <c r="B94" t="n">
-        <v>10.16247919201729</v>
-      </c>
-      <c r="C94" t="n">
-        <v>-5.952375145557596</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>2401750016</v>
-      </c>
-      <c r="B95" t="n">
-        <v>10.23827483064315</v>
-      </c>
-      <c r="C95" t="n">
-        <v>-5.569754170700219</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>2426500096</v>
-      </c>
-      <c r="B96" t="n">
-        <v>9.972450625304663</v>
-      </c>
-      <c r="C96" t="n">
-        <v>-5.694441532158958</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>2451249920</v>
-      </c>
-      <c r="B97" t="n">
-        <v>9.856031709475278</v>
-      </c>
-      <c r="C97" t="n">
-        <v>-5.493233390577252</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>2476000000</v>
-      </c>
-      <c r="B98" t="n">
-        <v>9.842956404535393</v>
-      </c>
-      <c r="C98" t="n">
-        <v>-5.413848370177824</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>2500750080</v>
-      </c>
-      <c r="B99" t="n">
-        <v>9.944431092912115</v>
-      </c>
-      <c r="C99" t="n">
-        <v>-5.207950547946954</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>2525499904</v>
-      </c>
-      <c r="B100" t="n">
-        <v>10.12535798648273</v>
-      </c>
-      <c r="C100" t="n">
-        <v>-5.165286555382686</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>2550249984</v>
-      </c>
-      <c r="B101" t="n">
-        <v>9.804319803098574</v>
-      </c>
-      <c r="C101" t="n">
-        <v>-5.172634167476225</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>2575000064</v>
-      </c>
-      <c r="B102" t="n">
-        <v>9.789909490616925</v>
-      </c>
-      <c r="C102" t="n">
-        <v>-5.034359380582702</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>2599749888</v>
-      </c>
-      <c r="B103" t="n">
-        <v>9.804274942897868</v>
-      </c>
-      <c r="C103" t="n">
-        <v>-5.09607361589028</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>2624499968</v>
-      </c>
-      <c r="B104" t="n">
-        <v>10.0508951617211</v>
-      </c>
-      <c r="C104" t="n">
-        <v>-4.88255946476324</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>2649250048</v>
-      </c>
-      <c r="B105" t="n">
-        <v>9.716332467329062</v>
-      </c>
-      <c r="C105" t="n">
-        <v>-4.96003358274778</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>2673999872</v>
-      </c>
-      <c r="B106" t="n">
-        <v>9.718762102238754</v>
-      </c>
-      <c r="C106" t="n">
-        <v>-4.773689335680348</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>2698749952</v>
-      </c>
-      <c r="B107" t="n">
-        <v>9.813152896391369</v>
-      </c>
-      <c r="C107" t="n">
-        <v>-4.707722898352446</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>2723500032</v>
-      </c>
-      <c r="B108" t="n">
-        <v>9.844120791343169</v>
-      </c>
-      <c r="C108" t="n">
-        <v>-4.833115536282288</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>2748250112</v>
-      </c>
-      <c r="B109" t="n">
-        <v>9.751607011479248</v>
-      </c>
-      <c r="C109" t="n">
-        <v>-4.628111066049036</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>2772999936</v>
-      </c>
-      <c r="B110" t="n">
-        <v>9.545827492405817</v>
-      </c>
-      <c r="C110" t="n">
-        <v>-4.54735936321842</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>2797750016</v>
-      </c>
-      <c r="B111" t="n">
-        <v>9.665882556023831</v>
-      </c>
-      <c r="C111" t="n">
-        <v>-4.708477174806688</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>2822500096</v>
-      </c>
-      <c r="B112" t="n">
-        <v>9.739492661016579</v>
-      </c>
-      <c r="C112" t="n">
-        <v>-4.641738539089349</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>2847249920</v>
-      </c>
-      <c r="B113" t="n">
-        <v>9.63627510497988</v>
-      </c>
-      <c r="C113" t="n">
-        <v>-4.327943120834171</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>2872000000</v>
-      </c>
-      <c r="B114" t="n">
-        <v>9.445531030350669</v>
-      </c>
-      <c r="C114" t="n">
-        <v>-4.259694192265195</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>2896750080</v>
-      </c>
-      <c r="B115" t="n">
-        <v>9.754227801244413</v>
-      </c>
-      <c r="C115" t="n">
-        <v>-4.668694114577252</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>2921499904</v>
-      </c>
-      <c r="B116" t="n">
-        <v>9.853140307430145</v>
-      </c>
-      <c r="C116" t="n">
-        <v>-4.413317706726784</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>2946249984</v>
-      </c>
-      <c r="B117" t="n">
-        <v>9.437126632317218</v>
-      </c>
-      <c r="C117" t="n">
-        <v>-4.060344743386565</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>2971000064</v>
-      </c>
-      <c r="B118" t="n">
-        <v>9.177822070874813</v>
-      </c>
-      <c r="C118" t="n">
-        <v>-4.067901435276915</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>2995749888</v>
-      </c>
-      <c r="B119" t="n">
-        <v>9.385847739072499</v>
-      </c>
-      <c r="C119" t="n">
-        <v>-4.292655940863484</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>3020499968</v>
-      </c>
-      <c r="B120" t="n">
-        <v>9.678939032505507</v>
-      </c>
-      <c r="C120" t="n">
-        <v>-4.260292508338359</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>3045250048</v>
-      </c>
-      <c r="B121" t="n">
-        <v>9.530137116925365</v>
-      </c>
-      <c r="C121" t="n">
-        <v>-4.141647108681841</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>3070000128</v>
-      </c>
-      <c r="B122" t="n">
-        <v>9.28473091465564</v>
-      </c>
-      <c r="C122" t="n">
-        <v>-3.942103894983001</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>3094749952</v>
-      </c>
-      <c r="B123" t="n">
-        <v>9.282721392212377</v>
-      </c>
-      <c r="C123" t="n">
-        <v>-4.11285545233866</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>3119500032</v>
-      </c>
-      <c r="B124" t="n">
-        <v>9.482779067871379</v>
-      </c>
-      <c r="C124" t="n">
-        <v>-4.059937255562057</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>3144250112</v>
-      </c>
-      <c r="B125" t="n">
-        <v>9.41751586945934</v>
-      </c>
-      <c r="C125" t="n">
-        <v>-3.982311925634417</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>3168999936</v>
-      </c>
-      <c r="B126" t="n">
-        <v>9.109048731910633</v>
-      </c>
-      <c r="C126" t="n">
-        <v>-3.708577546663359</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>3193750016</v>
-      </c>
-      <c r="B127" t="n">
-        <v>8.950536133893447</v>
-      </c>
-      <c r="C127" t="n">
-        <v>-4.011916254162654</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>3218500096</v>
-      </c>
-      <c r="B128" t="n">
-        <v>9.455820883011141</v>
-      </c>
-      <c r="C128" t="n">
-        <v>-3.969779331964319</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>3243249920</v>
-      </c>
-      <c r="B129" t="n">
-        <v>9.365329477451144</v>
-      </c>
-      <c r="C129" t="n">
-        <v>-3.797895143557608</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>3268000000</v>
-      </c>
-      <c r="B130" t="n">
-        <v>9.081199223113941</v>
-      </c>
-      <c r="C130" t="n">
-        <v>-3.563390996594386</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>3292750080</v>
-      </c>
-      <c r="B131" t="n">
-        <v>9.106494332035243</v>
-      </c>
-      <c r="C131" t="n">
-        <v>-3.734086584644347</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>3317499904</v>
-      </c>
-      <c r="B132" t="n">
-        <v>9.287229228089608</v>
-      </c>
-      <c r="C132" t="n">
-        <v>-3.984221614438097</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>3342249984</v>
-      </c>
-      <c r="B133" t="n">
-        <v>9.27140633402197</v>
-      </c>
-      <c r="C133" t="n">
-        <v>-3.894591293642931</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="n">
-        <v>3367000064</v>
-      </c>
-      <c r="B134" t="n">
-        <v>9.05050976125338</v>
-      </c>
-      <c r="C134" t="n">
-        <v>-3.42739642858187</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="n">
-        <v>3391749888</v>
-      </c>
-      <c r="B135" t="n">
-        <v>8.953287479630603</v>
-      </c>
-      <c r="C135" t="n">
-        <v>-3.429053913735959</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="n">
-        <v>3416499968</v>
-      </c>
-      <c r="B136" t="n">
-        <v>8.982722357671092</v>
-      </c>
-      <c r="C136" t="n">
-        <v>-3.815667310616674</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="n">
-        <v>3441250048</v>
-      </c>
-      <c r="B137" t="n">
-        <v>9.117858183009869</v>
-      </c>
-      <c r="C137" t="n">
-        <v>-3.590560519781282</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="n">
-        <v>3465999872</v>
-      </c>
-      <c r="B138" t="n">
-        <v>9.170288570193335</v>
-      </c>
-      <c r="C138" t="n">
-        <v>-3.262621530567833</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="n">
-        <v>3490749952</v>
-      </c>
-      <c r="B139" t="n">
-        <v>8.884394528167146</v>
-      </c>
-      <c r="C139" t="n">
-        <v>-3.233115890359501</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="n">
-        <v>3515500032</v>
-      </c>
-      <c r="B140" t="n">
-        <v>8.765637742889934</v>
-      </c>
-      <c r="C140" t="n">
-        <v>-3.410517241083158</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="n">
-        <v>3540250112</v>
-      </c>
-      <c r="B141" t="n">
-        <v>8.776632526283493</v>
-      </c>
-      <c r="C141" t="n">
-        <v>-3.563033919492663</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="n">
-        <v>3564999936</v>
-      </c>
-      <c r="B142" t="n">
-        <v>8.96559643985076</v>
-      </c>
-      <c r="C142" t="n">
-        <v>-3.176129362594442</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="n">
-        <v>3589750016</v>
-      </c>
-      <c r="B143" t="n">
-        <v>8.823139326766196</v>
-      </c>
-      <c r="C143" t="n">
-        <v>-2.940759656334442</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="n">
-        <v>3614500096</v>
-      </c>
-      <c r="B144" t="n">
-        <v>8.697935617194263</v>
-      </c>
-      <c r="C144" t="n">
-        <v>-3.262728366838894</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="n">
-        <v>3639249920</v>
-      </c>
-      <c r="B145" t="n">
-        <v>8.721718474962669</v>
-      </c>
-      <c r="C145" t="n">
-        <v>-3.305062284052587</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="n">
-        <v>3664000000</v>
-      </c>
-      <c r="B146" t="n">
-        <v>8.836768543257032</v>
-      </c>
-      <c r="C146" t="n">
-        <v>-2.933346342795907</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="n">
-        <v>3688750080</v>
-      </c>
-      <c r="B147" t="n">
-        <v>8.733794541358696</v>
-      </c>
-      <c r="C147" t="n">
-        <v>-2.593044297524844</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="n">
-        <v>3713499904</v>
-      </c>
-      <c r="B148" t="n">
-        <v>8.562251263808317</v>
-      </c>
-      <c r="C148" t="n">
-        <v>-3.038568171554189</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="n">
-        <v>3738249984</v>
-      </c>
-      <c r="B149" t="n">
-        <v>8.502411149350808</v>
-      </c>
-      <c r="C149" t="n">
-        <v>-3.091620090614977</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>3763000064</v>
-      </c>
-      <c r="B150" t="n">
-        <v>8.611878294686646</v>
-      </c>
-      <c r="C150" t="n">
-        <v>-2.858135132553959</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="n">
-        <v>3787749888</v>
-      </c>
-      <c r="B151" t="n">
-        <v>8.776542816797619</v>
-      </c>
-      <c r="C151" t="n">
-        <v>-2.612951149888553</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="n">
-        <v>3812499968</v>
-      </c>
-      <c r="B152" t="n">
-        <v>8.565009721913979</v>
-      </c>
-      <c r="C152" t="n">
-        <v>-2.596948954871566</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="n">
-        <v>3837250048</v>
-      </c>
-      <c r="B153" t="n">
-        <v>8.445186722664726</v>
-      </c>
-      <c r="C153" t="n">
-        <v>-2.884263164613334</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="n">
-        <v>3862000128</v>
-      </c>
-      <c r="B154" t="n">
-        <v>8.593445047883677</v>
-      </c>
-      <c r="C154" t="n">
-        <v>-2.62904158876536</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="n">
-        <v>3886749952</v>
-      </c>
-      <c r="B155" t="n">
-        <v>8.646723792664613</v>
-      </c>
-      <c r="C155" t="n">
-        <v>-2.337829329427834</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="n">
-        <v>3911500032</v>
-      </c>
-      <c r="B156" t="n">
-        <v>8.418027225440049</v>
-      </c>
-      <c r="C156" t="n">
-        <v>-2.533377490856098</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="n">
-        <v>3936250112</v>
-      </c>
-      <c r="B157" t="n">
-        <v>8.337555241534531</v>
-      </c>
-      <c r="C157" t="n">
-        <v>-2.614609863796525</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="n">
-        <v>3960999936</v>
-      </c>
-      <c r="B158" t="n">
-        <v>8.552523030683187</v>
-      </c>
-      <c r="C158" t="n">
-        <v>-2.532927314423216</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="n">
-        <v>3985750016</v>
-      </c>
-      <c r="B159" t="n">
-        <v>8.655463484472731</v>
-      </c>
-      <c r="C159" t="n">
-        <v>-2.33405914279598</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="n">
-        <v>4010500096</v>
-      </c>
-      <c r="B160" t="n">
-        <v>8.544066513455626</v>
-      </c>
-      <c r="C160" t="n">
-        <v>-2.254238420495982</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="n">
-        <v>4035249920</v>
-      </c>
-      <c r="B161" t="n">
-        <v>8.23391620545903</v>
-      </c>
-      <c r="C161" t="n">
-        <v>-2.459507489407886</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="n">
-        <v>4060000000</v>
-      </c>
-      <c r="B162" t="n">
-        <v>8.377635414885498</v>
-      </c>
-      <c r="C162" t="n">
-        <v>-2.406144222875692</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="n">
-        <v>4084750080</v>
-      </c>
-      <c r="B163" t="n">
-        <v>8.559226809805242</v>
-      </c>
-      <c r="C163" t="n">
-        <v>-2.292276291759492</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="n">
-        <v>4109499904</v>
-      </c>
-      <c r="B164" t="n">
-        <v>8.541204529216692</v>
-      </c>
-      <c r="C164" t="n">
-        <v>-2.152637170043839</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="n">
-        <v>4134249984</v>
-      </c>
-      <c r="B165" t="n">
-        <v>8.18875859570092</v>
-      </c>
-      <c r="C165" t="n">
-        <v>-2.126070779567857</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="n">
-        <v>4159000064</v>
-      </c>
-      <c r="B166" t="n">
-        <v>8.273351811745403</v>
-      </c>
-      <c r="C166" t="n">
-        <v>-2.329626160457573</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="n">
-        <v>4183749888</v>
-      </c>
-      <c r="B167" t="n">
-        <v>8.548411838314774</v>
-      </c>
-      <c r="C167" t="n">
-        <v>-2.106795597819235</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="n">
-        <v>4208499968</v>
-      </c>
-      <c r="B168" t="n">
-        <v>8.344884112090103</v>
-      </c>
-      <c r="C168" t="n">
-        <v>-1.928550455539638</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="n">
-        <v>4233250048</v>
-      </c>
-      <c r="B169" t="n">
-        <v>8.242560657979352</v>
-      </c>
-      <c r="C169" t="n">
-        <v>-2.046793534816498</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="n">
-        <v>4257999872</v>
-      </c>
-      <c r="B170" t="n">
-        <v>8.272988904241473</v>
-      </c>
-      <c r="C170" t="n">
-        <v>-2.117247811402554</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="n">
-        <v>4282749952</v>
-      </c>
-      <c r="B171" t="n">
-        <v>8.524513085448602</v>
-      </c>
-      <c r="C171" t="n">
-        <v>-1.958892221476214</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="n">
-        <v>4307500032</v>
-      </c>
-      <c r="B172" t="n">
-        <v>8.517893862848378</v>
-      </c>
-      <c r="C172" t="n">
-        <v>-1.870509859397349</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="n">
-        <v>4332250112</v>
-      </c>
-      <c r="B173" t="n">
-        <v>8.320769042826599</v>
-      </c>
-      <c r="C173" t="n">
-        <v>-1.984500527912919</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="n">
-        <v>4357000192</v>
-      </c>
-      <c r="B174" t="n">
-        <v>8.176643252422465</v>
-      </c>
-      <c r="C174" t="n">
-        <v>-1.920364546711881</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="n">
-        <v>4381749760</v>
-      </c>
-      <c r="B175" t="n">
-        <v>8.423825807199199</v>
-      </c>
-      <c r="C175" t="n">
-        <v>-1.814204214557213</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="n">
-        <v>4406499840</v>
-      </c>
-      <c r="B176" t="n">
-        <v>8.378717993214003</v>
-      </c>
-      <c r="C176" t="n">
-        <v>-1.69057688315351</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="n">
-        <v>4431249920</v>
-      </c>
-      <c r="B177" t="n">
-        <v>8.191791103144528</v>
-      </c>
-      <c r="C177" t="n">
-        <v>-1.59837280928488</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="n">
-        <v>4456000000</v>
-      </c>
-      <c r="B178" t="n">
-        <v>8.25778499291785</v>
-      </c>
-      <c r="C178" t="n">
-        <v>-1.827081943505573</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="n">
-        <v>4480750080</v>
-      </c>
-      <c r="B179" t="n">
-        <v>8.370542418561048</v>
-      </c>
-      <c r="C179" t="n">
-        <v>-1.713200409148403</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="n">
-        <v>4505500160</v>
-      </c>
-      <c r="B180" t="n">
-        <v>8.486746310580727</v>
-      </c>
-      <c r="C180" t="n">
-        <v>-1.604474685098374</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="n">
-        <v>4530250240</v>
-      </c>
-      <c r="B181" t="n">
-        <v>8.30760111077972</v>
-      </c>
-      <c r="C181" t="n">
-        <v>-1.558760860980348</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="n">
-        <v>4554999808</v>
-      </c>
-      <c r="B182" t="n">
-        <v>8.22244157504727</v>
-      </c>
-      <c r="C182" t="n">
-        <v>-1.626940591871655</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="n">
-        <v>4579749888</v>
-      </c>
-      <c r="B183" t="n">
-        <v>8.352204092287769</v>
-      </c>
-      <c r="C183" t="n">
-        <v>-1.504647122431049</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="n">
-        <v>4604499968</v>
-      </c>
-      <c r="B184" t="n">
-        <v>8.38179654087519</v>
-      </c>
-      <c r="C184" t="n">
-        <v>-1.492120306398723</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="n">
-        <v>4629250048</v>
-      </c>
-      <c r="B185" t="n">
-        <v>8.22261697453661</v>
-      </c>
-      <c r="C185" t="n">
-        <v>-1.484595208445542</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="n">
-        <v>4654000128</v>
-      </c>
-      <c r="B186" t="n">
-        <v>8.155037253233345</v>
-      </c>
-      <c r="C186" t="n">
-        <v>-1.479818364310955</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="n">
-        <v>4678750208</v>
-      </c>
-      <c r="B187" t="n">
-        <v>8.124346771884293</v>
-      </c>
-      <c r="C187" t="n">
-        <v>-1.475288807907069</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="n">
-        <v>4703499776</v>
-      </c>
-      <c r="B188" t="n">
-        <v>8.245911672098218</v>
-      </c>
-      <c r="C188" t="n">
-        <v>-1.381550109224551</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="n">
-        <v>4728249856</v>
-      </c>
-      <c r="B189" t="n">
-        <v>8.154833505892018</v>
-      </c>
-      <c r="C189" t="n">
-        <v>-1.257176939442614</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="n">
-        <v>4752999936</v>
-      </c>
-      <c r="B190" t="n">
-        <v>8.03701987364035</v>
-      </c>
-      <c r="C190" t="n">
-        <v>-1.338316075837762</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="n">
-        <v>4777750016</v>
-      </c>
-      <c r="B191" t="n">
-        <v>8.091683030365962</v>
-      </c>
-      <c r="C191" t="n">
-        <v>-1.363057343590969</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="n">
-        <v>4802500096</v>
-      </c>
-      <c r="B192" t="n">
-        <v>8.218396990209516</v>
-      </c>
-      <c r="C192" t="n">
-        <v>-1.303963174976585</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="n">
-        <v>4827250176</v>
-      </c>
-      <c r="B193" t="n">
-        <v>8.16781510356782</v>
-      </c>
-      <c r="C193" t="n">
-        <v>-1.140677871151592</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="n">
-        <v>4851999744</v>
-      </c>
-      <c r="B194" t="n">
-        <v>7.990620846475736</v>
-      </c>
-      <c r="C194" t="n">
-        <v>-1.211348358435117</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="n">
-        <v>4876749824</v>
-      </c>
-      <c r="B195" t="n">
-        <v>8.042015553565999</v>
-      </c>
-      <c r="C195" t="n">
-        <v>-1.20523797560135</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="n">
-        <v>4901499904</v>
-      </c>
-      <c r="B196" t="n">
-        <v>8.079896021521984</v>
-      </c>
-      <c r="C196" t="n">
-        <v>-1.063164167373586</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="n">
-        <v>4926249984</v>
-      </c>
-      <c r="B197" t="n">
-        <v>8.212310200226099</v>
-      </c>
-      <c r="C197" t="n">
-        <v>-1.043995141154058</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>4951000064</v>
-      </c>
-      <c r="B198" t="n">
-        <v>8.033970292534839</v>
-      </c>
-      <c r="C198" t="n">
-        <v>-1.018783140790827</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="n">
-        <v>4975750144</v>
-      </c>
-      <c r="B199" t="n">
-        <v>7.920037847181139</v>
-      </c>
-      <c r="C199" t="n">
-        <v>-1.099359790849523</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="n">
-        <v>5000500224</v>
-      </c>
-      <c r="B200" t="n">
-        <v>8.189052574331424</v>
-      </c>
-      <c r="C200" t="n">
-        <v>-1.059340773944246</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="n">
-        <v>5025249792</v>
-      </c>
-      <c r="B201" t="n">
-        <v>8.389002452320817</v>
-      </c>
-      <c r="C201" t="n">
-        <v>-0.9611653785201977</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="n">
-        <v>5049999872</v>
-      </c>
-      <c r="B202" t="n">
-        <v>8.040493940887366</v>
-      </c>
-      <c r="C202" t="n">
-        <v>-1.020602145729635</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="n">
-        <v>5074749952</v>
-      </c>
-      <c r="B203" t="n">
-        <v>7.894758198262957</v>
-      </c>
-      <c r="C203" t="n">
-        <v>-0.9379599608135671</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="n">
-        <v>5099500032</v>
-      </c>
-      <c r="B204" t="n">
-        <v>7.952371197000969</v>
-      </c>
-      <c r="C204" t="n">
-        <v>-0.8334852033857655</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="n">
-        <v>5124250112</v>
-      </c>
-      <c r="B205" t="n">
-        <v>7.979679008482798</v>
-      </c>
-      <c r="C205" t="n">
-        <v>-0.7856633559036036</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="n">
-        <v>5149000192</v>
-      </c>
-      <c r="B206" t="n">
-        <v>7.965362417435135</v>
-      </c>
-      <c r="C206" t="n">
-        <v>-0.7131939613099685</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="n">
-        <v>5173749760</v>
-      </c>
-      <c r="B207" t="n">
-        <v>7.870607078539488</v>
-      </c>
-      <c r="C207" t="n">
-        <v>-0.7796464128908398</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="n">
-        <v>5198499840</v>
-      </c>
-      <c r="B208" t="n">
-        <v>8.02473612836901</v>
-      </c>
-      <c r="C208" t="n">
-        <v>-0.7413451545199989</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="n">
-        <v>5223249920</v>
-      </c>
-      <c r="B209" t="n">
-        <v>8.033109241765178</v>
-      </c>
-      <c r="C209" t="n">
-        <v>-0.7730457952683559</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="n">
-        <v>5248000000</v>
-      </c>
-      <c r="B210" t="n">
-        <v>7.900171093725759</v>
-      </c>
-      <c r="C210" t="n">
-        <v>-0.7304051847195284</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
-        <v>5272750080</v>
-      </c>
-      <c r="B211" t="n">
-        <v>7.913226559330461</v>
-      </c>
-      <c r="C211" t="n">
-        <v>-0.6576984336372489</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="n">
-        <v>5297500160</v>
-      </c>
-      <c r="B212" t="n">
-        <v>7.754491058280469</v>
-      </c>
-      <c r="C212" t="n">
-        <v>-0.7154104352363129</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="n">
-        <v>5322250240</v>
-      </c>
-      <c r="B213" t="n">
-        <v>7.970356163321299</v>
-      </c>
-      <c r="C213" t="n">
-        <v>-0.6747536172569896</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="n">
-        <v>5346999808</v>
-      </c>
-      <c r="B214" t="n">
-        <v>7.840516177733284</v>
-      </c>
-      <c r="C214" t="n">
-        <v>-0.6083237319111996</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="n">
-        <v>5371749888</v>
-      </c>
-      <c r="B215" t="n">
-        <v>7.711896307702933</v>
-      </c>
-      <c r="C215" t="n">
-        <v>-0.488338930548317</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="n">
-        <v>5396499968</v>
-      </c>
-      <c r="B216" t="n">
-        <v>7.826233417351557</v>
-      </c>
-      <c r="C216" t="n">
-        <v>-0.7463165574319359</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="n">
-        <v>5421250048</v>
-      </c>
-      <c r="B217" t="n">
-        <v>7.889475884651581</v>
-      </c>
-      <c r="C217" t="n">
-        <v>-0.638806507911812</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="n">
-        <v>5446000128</v>
-      </c>
-      <c r="B218" t="n">
-        <v>7.950262135691817</v>
-      </c>
-      <c r="C218" t="n">
-        <v>-0.5713731877358695</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="n">
-        <v>5470750208</v>
-      </c>
-      <c r="B219" t="n">
-        <v>7.844487274665369</v>
-      </c>
-      <c r="C219" t="n">
-        <v>-0.617731454634441</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="n">
-        <v>5495499776</v>
-      </c>
-      <c r="B220" t="n">
-        <v>7.686698270190702</v>
-      </c>
-      <c r="C220" t="n">
-        <v>-0.4664877866430046</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="n">
-        <v>5520249856</v>
-      </c>
-      <c r="B221" t="n">
-        <v>7.921858074168243</v>
-      </c>
-      <c r="C221" t="n">
-        <v>-0.4732964550962344</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
-        <v>5544999936</v>
-      </c>
-      <c r="B222" t="n">
-        <v>7.815804912355889</v>
-      </c>
-      <c r="C222" t="n">
-        <v>-0.4810476606994555</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
-        <v>5569750016</v>
-      </c>
-      <c r="B223" t="n">
-        <v>7.731988144913024</v>
-      </c>
-      <c r="C223" t="n">
-        <v>-0.6600967250477169</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="n">
-        <v>5594500096</v>
-      </c>
-      <c r="B224" t="n">
-        <v>7.81902654688333</v>
-      </c>
-      <c r="C224" t="n">
-        <v>-0.4381136806508453</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="n">
-        <v>5619250176</v>
-      </c>
-      <c r="B225" t="n">
-        <v>7.796642837828772</v>
-      </c>
-      <c r="C225" t="n">
-        <v>-0.3677405863323965</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="n">
-        <v>5644000256</v>
-      </c>
-      <c r="B226" t="n">
-        <v>7.808582349099994</v>
-      </c>
-      <c r="C226" t="n">
-        <v>-0.5467254959804035</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="n">
-        <v>5668749824</v>
-      </c>
-      <c r="B227" t="n">
-        <v>7.893320365267656</v>
-      </c>
-      <c r="C227" t="n">
-        <v>-0.2115557373702228</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="n">
-        <v>5693499904</v>
-      </c>
-      <c r="B228" t="n">
-        <v>7.778698197334518</v>
-      </c>
-      <c r="C228" t="n">
-        <v>-0.3722399326792862</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="n">
-        <v>5718249984</v>
-      </c>
-      <c r="B229" t="n">
-        <v>7.779009499865206</v>
-      </c>
-      <c r="C229" t="n">
-        <v>-0.4315928759262112</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="n">
-        <v>5743000064</v>
-      </c>
-      <c r="B230" t="n">
-        <v>7.714321811882093</v>
-      </c>
-      <c r="C230" t="n">
-        <v>-0.3235743087902513</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="n">
-        <v>5767750144</v>
-      </c>
-      <c r="B231" t="n">
-        <v>7.764102154264756</v>
-      </c>
-      <c r="C231" t="n">
-        <v>-0.2817217688772281</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="n">
-        <v>5792500224</v>
-      </c>
-      <c r="B232" t="n">
-        <v>7.764184134891458</v>
-      </c>
-      <c r="C232" t="n">
-        <v>-0.2803239091151027</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="n">
-        <v>5817249792</v>
-      </c>
-      <c r="B233" t="n">
-        <v>7.833167275402305</v>
-      </c>
-      <c r="C233" t="n">
-        <v>-0.1727879020181557</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="n">
-        <v>5841999872</v>
-      </c>
-      <c r="B234" t="n">
-        <v>7.891506998435941</v>
-      </c>
-      <c r="C234" t="n">
-        <v>-0.1142497696263653</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="n">
-        <v>5866749952</v>
-      </c>
-      <c r="B235" t="n">
-        <v>7.706841591844696</v>
-      </c>
-      <c r="C235" t="n">
-        <v>-0.0997526311494388</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="n">
-        <v>5891500032</v>
-      </c>
-      <c r="B236" t="n">
-        <v>7.717922477937884</v>
-      </c>
-      <c r="C236" t="n">
-        <v>-0.04641963276833543</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="n">
-        <v>5916250112</v>
-      </c>
-      <c r="B237" t="n">
-        <v>7.779365110171778</v>
-      </c>
-      <c r="C237" t="n">
-        <v>0.05747800848424667</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="n">
-        <v>5941000192</v>
-      </c>
-      <c r="B238" t="n">
-        <v>7.625706424096238</v>
-      </c>
-      <c r="C238" t="n">
-        <v>0.01573807260481152</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="n">
-        <v>5965749760</v>
-      </c>
-      <c r="B239" t="n">
-        <v>7.748893367703409</v>
-      </c>
-      <c r="C239" t="n">
-        <v>-0.09791363086652971</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="n">
-        <v>5990499840</v>
-      </c>
-      <c r="B240" t="n">
-        <v>7.68436447253436</v>
-      </c>
-      <c r="C240" t="n">
-        <v>0.04269656701476572</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="n">
-        <v>6015249920</v>
-      </c>
-      <c r="B241" t="n">
-        <v>7.66795257325334</v>
-      </c>
-      <c r="C241" t="n">
-        <v>0.02847585899427785</v>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="n">
-        <v>6040000000</v>
-      </c>
-      <c r="B242" t="n">
-        <v>7.679389283726953</v>
-      </c>
-      <c r="C242" t="n">
-        <v>-0.04877276038813489</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="n">
-        <v>6064750080</v>
-      </c>
-      <c r="B243" t="n">
-        <v>7.718127214250281</v>
-      </c>
-      <c r="C243" t="n">
-        <v>-0.004910503719296116</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="n">
-        <v>6089500160</v>
-      </c>
-      <c r="B244" t="n">
-        <v>7.741129675109439</v>
-      </c>
-      <c r="C244" t="n">
-        <v>0.17594940252506</v>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="n">
-        <v>6114250240</v>
-      </c>
-      <c r="B245" t="n">
-        <v>7.647817268134406</v>
-      </c>
-      <c r="C245" t="n">
-        <v>0.04674680564660507</v>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="n">
-        <v>6138999808</v>
-      </c>
-      <c r="B246" t="n">
-        <v>7.648474698602224</v>
-      </c>
-      <c r="C246" t="n">
-        <v>0.07932045645280067</v>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="n">
-        <v>6163749888</v>
-      </c>
-      <c r="B247" t="n">
-        <v>7.669412375355407</v>
-      </c>
-      <c r="C247" t="n">
-        <v>0.2010980954057473</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="n">
-        <v>6188499968</v>
-      </c>
-      <c r="B248" t="n">
-        <v>7.437768533845122</v>
-      </c>
-      <c r="C248" t="n">
-        <v>0.3775768260776868</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="n">
-        <v>6213250048</v>
-      </c>
-      <c r="B249" t="n">
-        <v>7.614107327368048</v>
-      </c>
-      <c r="C249" t="n">
-        <v>0.259787871018562</v>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="n">
-        <v>6238000128</v>
-      </c>
-      <c r="B250" t="n">
-        <v>7.532070176770159</v>
-      </c>
-      <c r="C250" t="n">
-        <v>0.1591443886106082</v>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="n">
-        <v>6262750208</v>
-      </c>
-      <c r="B251" t="n">
-        <v>7.546529579721349</v>
-      </c>
-      <c r="C251" t="n">
-        <v>0.2090542122654226</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="n">
-        <v>6287499776</v>
-      </c>
-      <c r="B252" t="n">
-        <v>7.368451159727107</v>
-      </c>
-      <c r="C252" t="n">
-        <v>0.2755826163139727</v>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="n">
-        <v>6312249856</v>
-      </c>
-      <c r="B253" t="n">
-        <v>7.483074901548966</v>
-      </c>
-      <c r="C253" t="n">
-        <v>0.2329548553156174</v>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="n">
-        <v>6336999936</v>
-      </c>
-      <c r="B254" t="n">
-        <v>7.466437123026918</v>
-      </c>
-      <c r="C254" t="n">
-        <v>0.259784663401858</v>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="n">
-        <v>6361750016</v>
-      </c>
-      <c r="B255" t="n">
-        <v>7.572502278657761</v>
-      </c>
-      <c r="C255" t="n">
-        <v>0.3064547835272812</v>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="n">
-        <v>6386500096</v>
-      </c>
-      <c r="B256" t="n">
-        <v>7.53384421913209</v>
-      </c>
-      <c r="C256" t="n">
-        <v>0.3988634992241558</v>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="n">
-        <v>6411250176</v>
-      </c>
-      <c r="B257" t="n">
-        <v>7.474213035769107</v>
-      </c>
-      <c r="C257" t="n">
-        <v>0.2456528474429142</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="n">
-        <v>6435999744</v>
-      </c>
-      <c r="B258" t="n">
-        <v>7.505603977116249</v>
-      </c>
-      <c r="C258" t="n">
-        <v>0.3264477339031733</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="n">
-        <v>6460749824</v>
-      </c>
-      <c r="B259" t="n">
-        <v>7.4517390751276</v>
-      </c>
-      <c r="C259" t="n">
-        <v>0.2363220827842177</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="n">
-        <v>6485499904</v>
-      </c>
-      <c r="B260" t="n">
-        <v>7.363262387450068</v>
-      </c>
-      <c r="C260" t="n">
-        <v>0.3466105794578481</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="n">
-        <v>6510249984</v>
-      </c>
-      <c r="B261" t="n">
-        <v>7.416615976414322</v>
-      </c>
-      <c r="C261" t="n">
-        <v>0.3898016861432146</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="n">
-        <v>6535000064</v>
-      </c>
-      <c r="B262" t="n">
-        <v>7.485606045534754</v>
-      </c>
-      <c r="C262" t="n">
-        <v>0.3906225532552662</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="n">
-        <v>6559750144</v>
-      </c>
-      <c r="B263" t="n">
-        <v>7.452715251487833</v>
-      </c>
-      <c r="C263" t="n">
-        <v>0.3912740924619666</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="n">
-        <v>6584500224</v>
-      </c>
-      <c r="B264" t="n">
-        <v>7.422865010001067</v>
-      </c>
-      <c r="C264" t="n">
-        <v>0.4249295879985122</v>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="n">
-        <v>6609249792</v>
-      </c>
-      <c r="B265" t="n">
-        <v>7.397687102454814</v>
-      </c>
-      <c r="C265" t="n">
-        <v>0.4807399827150091</v>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="n">
-        <v>6633999872</v>
-      </c>
-      <c r="B266" t="n">
-        <v>7.46963324776604</v>
-      </c>
-      <c r="C266" t="n">
-        <v>0.3756048695863206</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="n">
-        <v>6658749952</v>
-      </c>
-      <c r="B267" t="n">
-        <v>7.408556756432689</v>
-      </c>
-      <c r="C267" t="n">
-        <v>0.4972813841756343</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="n">
-        <v>6683500032</v>
-      </c>
-      <c r="B268" t="n">
-        <v>7.440185987881788</v>
-      </c>
-      <c r="C268" t="n">
-        <v>0.5724489516855018</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="n">
-        <v>6708250112</v>
-      </c>
-      <c r="B269" t="n">
-        <v>7.398378838231486</v>
-      </c>
-      <c r="C269" t="n">
-        <v>0.5134519422702672</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="n">
-        <v>6733000192</v>
-      </c>
-      <c r="B270" t="n">
-        <v>7.331608509524218</v>
-      </c>
-      <c r="C270" t="n">
-        <v>0.4396253677485474</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="n">
-        <v>6757749760</v>
-      </c>
-      <c r="B271" t="n">
-        <v>7.410489845136965</v>
-      </c>
-      <c r="C271" t="n">
-        <v>0.6208876505700452</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="n">
-        <v>6782499840</v>
-      </c>
-      <c r="B272" t="n">
-        <v>7.301973163655304</v>
-      </c>
-      <c r="C272" t="n">
-        <v>0.5659049919358136</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="n">
-        <v>6807249920</v>
-      </c>
-      <c r="B273" t="n">
-        <v>7.419293546242781</v>
-      </c>
-      <c r="C273" t="n">
-        <v>0.551411486681187</v>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="n">
-        <v>6832000000</v>
-      </c>
-      <c r="B274" t="n">
-        <v>7.418723778303848</v>
-      </c>
-      <c r="C274" t="n">
-        <v>0.4960509258925314</v>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="n">
-        <v>6856750080</v>
-      </c>
-      <c r="B275" t="n">
-        <v>7.348031504683714</v>
-      </c>
-      <c r="C275" t="n">
-        <v>0.5914981435255594</v>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="n">
-        <v>6881500160</v>
-      </c>
-      <c r="B276" t="n">
-        <v>7.307624250927517</v>
-      </c>
-      <c r="C276" t="n">
-        <v>0.6966307513797695</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="n">
-        <v>6906250240</v>
-      </c>
-      <c r="B277" t="n">
-        <v>7.234529511835731</v>
-      </c>
-      <c r="C277" t="n">
-        <v>0.6912212979735537</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="n">
-        <v>6930999808</v>
-      </c>
-      <c r="B278" t="n">
-        <v>7.197332573990923</v>
-      </c>
-      <c r="C278" t="n">
-        <v>0.690321514666359</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="n">
-        <v>6955749888</v>
-      </c>
-      <c r="B279" t="n">
-        <v>7.264879786642605</v>
-      </c>
-      <c r="C279" t="n">
-        <v>0.7163739196745901</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="n">
-        <v>6980499968</v>
-      </c>
-      <c r="B280" t="n">
-        <v>7.298148766064447</v>
-      </c>
-      <c r="C280" t="n">
-        <v>0.7358033989903078</v>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="n">
-        <v>7005250048</v>
-      </c>
-      <c r="B281" t="n">
-        <v>7.243919929332294</v>
-      </c>
-      <c r="C281" t="n">
-        <v>0.7778916820159381</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="n">
-        <v>7030000128</v>
-      </c>
-      <c r="B282" t="n">
-        <v>7.326775188930108</v>
-      </c>
-      <c r="C282" t="n">
-        <v>0.6486082624716764</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="n">
-        <v>7054750208</v>
-      </c>
-      <c r="B283" t="n">
-        <v>7.165510226866488</v>
-      </c>
-      <c r="C283" t="n">
-        <v>0.8615080037965581</v>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="n">
-        <v>7079499776</v>
-      </c>
-      <c r="B284" t="n">
-        <v>7.170483566407997</v>
-      </c>
-      <c r="C284" t="n">
-        <v>0.7375733828854687</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="n">
-        <v>7104249856</v>
-      </c>
-      <c r="B285" t="n">
-        <v>7.129425415738974</v>
-      </c>
-      <c r="C285" t="n">
-        <v>0.8210343417126466</v>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="n">
-        <v>7128999936</v>
-      </c>
-      <c r="B286" t="n">
-        <v>7.280464562024951</v>
-      </c>
-      <c r="C286" t="n">
-        <v>0.8019235700485694</v>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="n">
-        <v>7153750016</v>
-      </c>
-      <c r="B287" t="n">
-        <v>7.217740140432348</v>
-      </c>
-      <c r="C287" t="n">
-        <v>0.7614325377471672</v>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="n">
-        <v>7178500096</v>
-      </c>
-      <c r="B288" t="n">
-        <v>7.242596880079327</v>
-      </c>
-      <c r="C288" t="n">
-        <v>0.8245907550852477</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="n">
-        <v>7203250176</v>
-      </c>
-      <c r="B289" t="n">
-        <v>7.108075450001955</v>
-      </c>
-      <c r="C289" t="n">
-        <v>0.8312728561888783</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="n">
-        <v>7228000256</v>
-      </c>
-      <c r="B290" t="n">
-        <v>7.194172720812429</v>
-      </c>
-      <c r="C290" t="n">
-        <v>0.9231219422695675</v>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="n">
-        <v>7252749824</v>
-      </c>
-      <c r="B291" t="n">
-        <v>7.206583446461708</v>
-      </c>
-      <c r="C291" t="n">
-        <v>0.8600478338987281</v>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="n">
-        <v>7277499904</v>
-      </c>
-      <c r="B292" t="n">
-        <v>7.235048599670455</v>
-      </c>
-      <c r="C292" t="n">
-        <v>0.8654797986560991</v>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="n">
-        <v>7302249984</v>
-      </c>
-      <c r="B293" t="n">
-        <v>7.184146196534968</v>
-      </c>
-      <c r="C293" t="n">
-        <v>0.8977114977890955</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="n">
-        <v>7327000064</v>
-      </c>
-      <c r="B294" t="n">
-        <v>7.04630502751724</v>
-      </c>
-      <c r="C294" t="n">
-        <v>1.006828503053901</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="n">
-        <v>7351750144</v>
-      </c>
-      <c r="B295" t="n">
-        <v>7.166461718314239</v>
-      </c>
-      <c r="C295" t="n">
-        <v>0.9617622032552072</v>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="n">
-        <v>7376500224</v>
-      </c>
-      <c r="B296" t="n">
-        <v>7.138968520823628</v>
-      </c>
-      <c r="C296" t="n">
-        <v>0.8581311880767254</v>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="n">
-        <v>7401249792</v>
-      </c>
-      <c r="B297" t="n">
-        <v>7.012660895303743</v>
-      </c>
-      <c r="C297" t="n">
-        <v>1.056004775250623</v>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="n">
-        <v>7425999872</v>
-      </c>
-      <c r="B298" t="n">
-        <v>6.95906450268095</v>
-      </c>
-      <c r="C298" t="n">
-        <v>1.041887387166441</v>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="n">
-        <v>7450749952</v>
-      </c>
-      <c r="B299" t="n">
-        <v>7.048009857785116</v>
-      </c>
-      <c r="C299" t="n">
-        <v>1.015269291686766</v>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="n">
-        <v>7475500032</v>
-      </c>
-      <c r="B300" t="n">
-        <v>7.03994756571583</v>
-      </c>
-      <c r="C300" t="n">
-        <v>1.010949313103525</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="n">
-        <v>7500250112</v>
-      </c>
-      <c r="B301" t="n">
-        <v>7.041848235632138</v>
-      </c>
-      <c r="C301" t="n">
-        <v>1.084573032706723</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="n">
-        <v>7525000192</v>
-      </c>
-      <c r="B302" t="n">
-        <v>7.005441000435687</v>
-      </c>
-      <c r="C302" t="n">
-        <v>1.037628877907195</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="n">
-        <v>7549749760</v>
-      </c>
-      <c r="B303" t="n">
-        <v>7.03468450125203</v>
-      </c>
-      <c r="C303" t="n">
-        <v>1.095791664957662</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="n">
-        <v>7574499840</v>
-      </c>
-      <c r="B304" t="n">
-        <v>7.010069004141656</v>
-      </c>
-      <c r="C304" t="n">
-        <v>0.9373887112906096</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="n">
-        <v>7599249920</v>
-      </c>
-      <c r="B305" t="n">
-        <v>7.078480125088885</v>
-      </c>
-      <c r="C305" t="n">
-        <v>1.09375286004771</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="n">
-        <v>7624000000</v>
-      </c>
-      <c r="B306" t="n">
-        <v>7.008980348147141</v>
-      </c>
-      <c r="C306" t="n">
-        <v>1.097211315313319</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="n">
-        <v>7648750080</v>
-      </c>
-      <c r="B307" t="n">
-        <v>6.973633285651244</v>
-      </c>
-      <c r="C307" t="n">
-        <v>1.139146577329695</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="n">
-        <v>7673500160</v>
-      </c>
-      <c r="B308" t="n">
-        <v>7.044442654767835</v>
-      </c>
-      <c r="C308" t="n">
-        <v>1.097494291326779</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="n">
-        <v>7698250240</v>
-      </c>
-      <c r="B309" t="n">
-        <v>7.027480231534241</v>
-      </c>
-      <c r="C309" t="n">
-        <v>1.20239083020655</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="n">
-        <v>7722999808</v>
-      </c>
-      <c r="B310" t="n">
-        <v>7.000897709201928</v>
-      </c>
-      <c r="C310" t="n">
-        <v>1.232509193028114</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="n">
-        <v>7747749888</v>
-      </c>
-      <c r="B311" t="n">
-        <v>6.934909430433021</v>
-      </c>
-      <c r="C311" t="n">
-        <v>1.149352485304587</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="n">
-        <v>7772499968</v>
-      </c>
-      <c r="B312" t="n">
-        <v>7.008931278271102</v>
-      </c>
-      <c r="C312" t="n">
-        <v>1.108897610679087</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="n">
-        <v>7797250048</v>
-      </c>
-      <c r="B313" t="n">
-        <v>6.910983436592697</v>
-      </c>
-      <c r="C313" t="n">
-        <v>1.185370531076724</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="n">
-        <v>7822000128</v>
-      </c>
-      <c r="B314" t="n">
-        <v>6.934060793693694</v>
-      </c>
-      <c r="C314" t="n">
-        <v>1.239023774398311</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="n">
-        <v>7846750208</v>
-      </c>
-      <c r="B315" t="n">
-        <v>6.907328100745009</v>
-      </c>
-      <c r="C315" t="n">
-        <v>1.274633487809477</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="n">
-        <v>7871499776</v>
-      </c>
-      <c r="B316" t="n">
-        <v>6.892664473372156</v>
-      </c>
-      <c r="C316" t="n">
-        <v>1.219399886182131</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="n">
-        <v>7896249856</v>
-      </c>
-      <c r="B317" t="n">
-        <v>6.858402020279093</v>
-      </c>
-      <c r="C317" t="n">
-        <v>1.219980740387313</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="n">
-        <v>7920999936</v>
-      </c>
-      <c r="B318" t="n">
-        <v>6.856742460797528</v>
-      </c>
-      <c r="C318" t="n">
-        <v>1.32531487723274</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="n">
-        <v>7945750016</v>
-      </c>
-      <c r="B319" t="n">
-        <v>6.851849298493187</v>
-      </c>
-      <c r="C319" t="n">
-        <v>1.170195645024831</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="n">
-        <v>7970500096</v>
-      </c>
-      <c r="B320" t="n">
-        <v>6.887476567131873</v>
-      </c>
-      <c r="C320" t="n">
-        <v>1.274291162929158</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="n">
-        <v>7995250176</v>
-      </c>
-      <c r="B321" t="n">
-        <v>6.77535563999018</v>
-      </c>
-      <c r="C321" t="n">
-        <v>1.315073743735766</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="n">
-        <v>8019999744</v>
-      </c>
-      <c r="B322" t="n">
-        <v>6.833453585625304</v>
-      </c>
-      <c r="C322" t="n">
-        <v>1.365523650949084</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="n">
-        <v>8044749824</v>
-      </c>
-      <c r="B323" t="n">
-        <v>6.714167002634865</v>
-      </c>
-      <c r="C323" t="n">
-        <v>1.401705785446649</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="n">
-        <v>8069499904</v>
-      </c>
-      <c r="B324" t="n">
-        <v>6.714727151336233</v>
-      </c>
-      <c r="C324" t="n">
-        <v>1.397557680892103</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="n">
-        <v>8094249984</v>
-      </c>
-      <c r="B325" t="n">
-        <v>6.769428381322276</v>
-      </c>
-      <c r="C325" t="n">
-        <v>1.33754474031561</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="n">
-        <v>8119000064</v>
-      </c>
-      <c r="B326" t="n">
-        <v>6.771261270226084</v>
-      </c>
-      <c r="C326" t="n">
-        <v>1.409191618827408</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="n">
-        <v>8143750144</v>
-      </c>
-      <c r="B327" t="n">
-        <v>6.700537330641788</v>
-      </c>
-      <c r="C327" t="n">
-        <v>1.477419965190289</v>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="n">
-        <v>8168500224</v>
-      </c>
-      <c r="B328" t="n">
-        <v>6.727533176406714</v>
-      </c>
-      <c r="C328" t="n">
-        <v>1.467867356451946</v>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="n">
-        <v>8193249792</v>
-      </c>
-      <c r="B329" t="n">
-        <v>6.726108583758727</v>
-      </c>
-      <c r="C329" t="n">
-        <v>1.42373892217413</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="n">
-        <v>8217999872</v>
-      </c>
-      <c r="B330" t="n">
-        <v>6.628525130037914</v>
-      </c>
-      <c r="C330" t="n">
-        <v>1.486547625069664</v>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="n">
-        <v>8242749952</v>
-      </c>
-      <c r="B331" t="n">
-        <v>6.638337699288381</v>
-      </c>
-      <c r="C331" t="n">
-        <v>1.49578242933554</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="n">
-        <v>8267500032</v>
-      </c>
-      <c r="B332" t="n">
-        <v>6.616525289896288</v>
-      </c>
-      <c r="C332" t="n">
-        <v>1.507074684899114</v>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="n">
-        <v>8292250112</v>
-      </c>
-      <c r="B333" t="n">
-        <v>6.64041508264901</v>
-      </c>
-      <c r="C333" t="n">
-        <v>1.45336511514982</v>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="n">
-        <v>8317000192</v>
-      </c>
-      <c r="B334" t="n">
-        <v>6.595323579779695</v>
-      </c>
-      <c r="C334" t="n">
-        <v>1.518705963382108</v>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="n">
-        <v>8341749760</v>
-      </c>
-      <c r="B335" t="n">
-        <v>6.666791980980361</v>
-      </c>
-      <c r="C335" t="n">
-        <v>1.475720412459697</v>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="n">
-        <v>8366499840</v>
-      </c>
-      <c r="B336" t="n">
-        <v>6.608739400701585</v>
-      </c>
-      <c r="C336" t="n">
-        <v>1.547359650003372</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="n">
-        <v>8391249920</v>
-      </c>
-      <c r="B337" t="n">
-        <v>6.620105079306629</v>
-      </c>
-      <c r="C337" t="n">
-        <v>1.546355044506029</v>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="n">
-        <v>8416000000</v>
-      </c>
-      <c r="B338" t="n">
-        <v>6.662311872389075</v>
-      </c>
-      <c r="C338" t="n">
-        <v>1.643398455648774</v>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="n">
-        <v>8440750080</v>
-      </c>
-      <c r="B339" t="n">
-        <v>6.529977845103203</v>
-      </c>
-      <c r="C339" t="n">
-        <v>1.562803009826643</v>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="n">
-        <v>8465500160</v>
-      </c>
-      <c r="B340" t="n">
-        <v>6.552030814801201</v>
-      </c>
-      <c r="C340" t="n">
-        <v>1.617405249574094</v>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="n">
-        <v>8490250240</v>
-      </c>
-      <c r="B341" t="n">
-        <v>6.619692629981381</v>
-      </c>
-      <c r="C341" t="n">
-        <v>1.569876804049213</v>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="n">
-        <v>8514999808</v>
-      </c>
-      <c r="B342" t="n">
-        <v>6.623846086078745</v>
-      </c>
-      <c r="C342" t="n">
-        <v>1.600999178695594</v>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="n">
-        <v>8539749888</v>
-      </c>
-      <c r="B343" t="n">
-        <v>6.548626247837262</v>
-      </c>
-      <c r="C343" t="n">
-        <v>1.591441879965479</v>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="n">
-        <v>8564499968</v>
-      </c>
-      <c r="B344" t="n">
-        <v>6.584045767827944</v>
-      </c>
-      <c r="C344" t="n">
-        <v>1.63895757336617</v>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="n">
-        <v>8589250048</v>
-      </c>
-      <c r="B345" t="n">
-        <v>6.582073646491416</v>
-      </c>
-      <c r="C345" t="n">
-        <v>1.685836328012386</v>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="n">
-        <v>8613999616</v>
-      </c>
-      <c r="B346" t="n">
-        <v>6.541015910214717</v>
-      </c>
-      <c r="C346" t="n">
-        <v>1.643476808203785</v>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="n">
-        <v>8638749696</v>
-      </c>
-      <c r="B347" t="n">
-        <v>6.577715887111197</v>
-      </c>
-      <c r="C347" t="n">
-        <v>1.670359789561328</v>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="n">
-        <v>8663499776</v>
-      </c>
-      <c r="B348" t="n">
-        <v>6.477529958599396</v>
-      </c>
-      <c r="C348" t="n">
-        <v>1.740324541012815</v>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="n">
-        <v>8688249856</v>
-      </c>
-      <c r="B349" t="n">
-        <v>6.409784295367029</v>
-      </c>
-      <c r="C349" t="n">
-        <v>1.692383071525758</v>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="n">
-        <v>8712999936</v>
-      </c>
-      <c r="B350" t="n">
-        <v>6.342742004072185</v>
-      </c>
-      <c r="C350" t="n">
-        <v>1.678425753412875</v>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="n">
-        <v>8737750016</v>
-      </c>
-      <c r="B351" t="n">
-        <v>6.461308441832617</v>
-      </c>
-      <c r="C351" t="n">
-        <v>1.74939450197449</v>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="n">
-        <v>8762500096</v>
-      </c>
-      <c r="B352" t="n">
-        <v>6.438553633287686</v>
-      </c>
-      <c r="C352" t="n">
-        <v>1.751527046032396</v>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" t="n">
-        <v>8787250176</v>
-      </c>
-      <c r="B353" t="n">
-        <v>6.39312299954337</v>
-      </c>
-      <c r="C353" t="n">
-        <v>1.839475469062469</v>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" t="n">
-        <v>8812000256</v>
-      </c>
-      <c r="B354" t="n">
-        <v>6.411241964414172</v>
-      </c>
-      <c r="C354" t="n">
-        <v>1.730845915313657</v>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" t="n">
-        <v>8836750336</v>
-      </c>
-      <c r="B355" t="n">
-        <v>6.40134307528418</v>
-      </c>
-      <c r="C355" t="n">
-        <v>1.877091345302959</v>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" t="n">
-        <v>8861500416</v>
-      </c>
-      <c r="B356" t="n">
-        <v>6.388248556616743</v>
-      </c>
-      <c r="C356" t="n">
-        <v>1.779142592173889</v>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" t="n">
-        <v>8886250496</v>
-      </c>
-      <c r="B357" t="n">
-        <v>6.333453016558248</v>
-      </c>
-      <c r="C357" t="n">
-        <v>1.722059880796841</v>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" t="n">
-        <v>8910999552</v>
-      </c>
-      <c r="B358" t="n">
-        <v>6.374687598212193</v>
-      </c>
-      <c r="C358" t="n">
-        <v>1.816980472826679</v>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" t="n">
-        <v>8935749632</v>
-      </c>
-      <c r="B359" t="n">
-        <v>6.381312488508325</v>
-      </c>
-      <c r="C359" t="n">
-        <v>1.793561387043376</v>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" t="n">
-        <v>8960499712</v>
-      </c>
-      <c r="B360" t="n">
-        <v>6.289490064461409</v>
-      </c>
-      <c r="C360" t="n">
-        <v>1.840074538253236</v>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" t="n">
-        <v>8985249792</v>
-      </c>
-      <c r="B361" t="n">
-        <v>6.322614240382088</v>
-      </c>
-      <c r="C361" t="n">
-        <v>1.806614464387402</v>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" t="n">
-        <v>9009999872</v>
-      </c>
-      <c r="B362" t="n">
-        <v>6.373748403940709</v>
-      </c>
-      <c r="C362" t="n">
-        <v>1.874213358103253</v>
-      </c>
-    </row>
-    <row r="363">
-      <c r="A363" t="n">
-        <v>9034749952</v>
-      </c>
-      <c r="B363" t="n">
-        <v>6.344627401500608</v>
-      </c>
-      <c r="C363" t="n">
-        <v>1.911680781536195</v>
-      </c>
-    </row>
-    <row r="364">
-      <c r="A364" t="n">
-        <v>9059500032</v>
-      </c>
-      <c r="B364" t="n">
-        <v>6.184884439157178</v>
-      </c>
-      <c r="C364" t="n">
-        <v>1.927562635358097</v>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" t="n">
-        <v>9084250112</v>
-      </c>
-      <c r="B365" t="n">
-        <v>6.27783567459946</v>
-      </c>
-      <c r="C365" t="n">
-        <v>1.949821165342938</v>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" t="n">
-        <v>9109000192</v>
-      </c>
-      <c r="B366" t="n">
-        <v>6.285482112258652</v>
-      </c>
-      <c r="C366" t="n">
-        <v>1.910040430854735</v>
-      </c>
-    </row>
-    <row r="367">
-      <c r="A367" t="n">
-        <v>9133750272</v>
-      </c>
-      <c r="B367" t="n">
-        <v>6.314664975196759</v>
-      </c>
-      <c r="C367" t="n">
-        <v>2.025158723540506</v>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" t="n">
-        <v>9158500352</v>
-      </c>
-      <c r="B368" t="n">
-        <v>6.266390515232805</v>
-      </c>
-      <c r="C368" t="n">
-        <v>2.012602141325211</v>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" t="n">
-        <v>9183250432</v>
-      </c>
-      <c r="B369" t="n">
-        <v>6.232920902412155</v>
-      </c>
-      <c r="C369" t="n">
-        <v>1.980566348345363</v>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" t="n">
-        <v>9208000512</v>
-      </c>
-      <c r="B370" t="n">
-        <v>6.288310231703266</v>
-      </c>
-      <c r="C370" t="n">
-        <v>2.003711401417057</v>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" t="n">
-        <v>9232749568</v>
-      </c>
-      <c r="B371" t="n">
-        <v>6.171990483588889</v>
-      </c>
-      <c r="C371" t="n">
-        <v>1.95860137587479</v>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" t="n">
-        <v>9257499648</v>
-      </c>
-      <c r="B372" t="n">
-        <v>6.201827842598419</v>
-      </c>
-      <c r="C372" t="n">
-        <v>1.977684058654432</v>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" t="n">
-        <v>9282249728</v>
-      </c>
-      <c r="B373" t="n">
-        <v>6.251860167201496</v>
-      </c>
-      <c r="C373" t="n">
-        <v>2.057471872367864</v>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="n">
-        <v>9306999808</v>
-      </c>
-      <c r="B374" t="n">
-        <v>6.270933518133191</v>
-      </c>
-      <c r="C374" t="n">
-        <v>2.053280828848885</v>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" t="n">
-        <v>9331749888</v>
-      </c>
-      <c r="B375" t="n">
-        <v>6.170630683361783</v>
-      </c>
-      <c r="C375" t="n">
-        <v>2.053612111330718</v>
-      </c>
-    </row>
-    <row r="376">
-      <c r="A376" t="n">
-        <v>9356499968</v>
-      </c>
-      <c r="B376" t="n">
-        <v>6.138469743509901</v>
-      </c>
-      <c r="C376" t="n">
-        <v>2.088106933979954</v>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="n">
-        <v>9381250048</v>
-      </c>
-      <c r="B377" t="n">
-        <v>6.128529035079088</v>
-      </c>
-      <c r="C377" t="n">
-        <v>2.060241950934504</v>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="n">
-        <v>9406000128</v>
-      </c>
-      <c r="B378" t="n">
-        <v>6.139354938504972</v>
-      </c>
-      <c r="C378" t="n">
-        <v>2.120156048318536</v>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" t="n">
-        <v>9430750208</v>
-      </c>
-      <c r="B379" t="n">
-        <v>6.177371059811144</v>
-      </c>
-      <c r="C379" t="n">
-        <v>2.092412459312974</v>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="n">
-        <v>9455500288</v>
-      </c>
-      <c r="B380" t="n">
-        <v>6.122144756263046</v>
-      </c>
-      <c r="C380" t="n">
-        <v>2.126707421795853</v>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" t="n">
-        <v>9480250368</v>
-      </c>
-      <c r="B381" t="n">
-        <v>6.145019278529535</v>
-      </c>
-      <c r="C381" t="n">
-        <v>2.078917721224459</v>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" t="n">
-        <v>9505000448</v>
-      </c>
-      <c r="B382" t="n">
-        <v>6.089308603868822</v>
-      </c>
-      <c r="C382" t="n">
-        <v>2.147934590383548</v>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="n">
-        <v>9529749504</v>
-      </c>
-      <c r="B383" t="n">
-        <v>6.146078487514702</v>
-      </c>
-      <c r="C383" t="n">
-        <v>2.182800603202633</v>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" t="n">
-        <v>9554499584</v>
-      </c>
-      <c r="B384" t="n">
-        <v>6.064503712272568</v>
-      </c>
-      <c r="C384" t="n">
-        <v>2.104941942964785</v>
-      </c>
-    </row>
-    <row r="385">
-      <c r="A385" t="n">
-        <v>9579249664</v>
-      </c>
-      <c r="B385" t="n">
-        <v>6.09869779084725</v>
-      </c>
-      <c r="C385" t="n">
-        <v>2.169376265069138</v>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" t="n">
-        <v>9603999744</v>
-      </c>
-      <c r="B386" t="n">
-        <v>6.03381471787557</v>
-      </c>
-      <c r="C386" t="n">
-        <v>2.239979891378208</v>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" t="n">
-        <v>9628749824</v>
-      </c>
-      <c r="B387" t="n">
-        <v>6.06467525299378</v>
-      </c>
-      <c r="C387" t="n">
-        <v>2.206803456178861</v>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" t="n">
-        <v>9653499904</v>
-      </c>
-      <c r="B388" t="n">
-        <v>6.058610369261382</v>
-      </c>
-      <c r="C388" t="n">
-        <v>2.209049839264075</v>
-      </c>
-    </row>
-    <row r="389">
-      <c r="A389" t="n">
-        <v>9678249984</v>
-      </c>
-      <c r="B389" t="n">
-        <v>6.061378366985931</v>
-      </c>
-      <c r="C389" t="n">
-        <v>2.259587729567568</v>
-      </c>
-    </row>
-    <row r="390">
-      <c r="A390" t="n">
-        <v>9703000064</v>
-      </c>
-      <c r="B390" t="n">
-        <v>6.036182428931069</v>
-      </c>
-      <c r="C390" t="n">
-        <v>2.177509862911986</v>
-      </c>
-    </row>
-    <row r="391">
-      <c r="A391" t="n">
-        <v>9727750144</v>
-      </c>
-      <c r="B391" t="n">
-        <v>5.921510857337021</v>
-      </c>
-      <c r="C391" t="n">
-        <v>2.228332071448128</v>
-      </c>
-    </row>
-    <row r="392">
-      <c r="A392" t="n">
-        <v>9752500224</v>
-      </c>
-      <c r="B392" t="n">
-        <v>5.945060201481436</v>
-      </c>
-      <c r="C392" t="n">
-        <v>2.25007214958638</v>
-      </c>
-    </row>
-    <row r="393">
-      <c r="A393" t="n">
-        <v>9777250304</v>
-      </c>
-      <c r="B393" t="n">
-        <v>5.986385340158884</v>
-      </c>
-      <c r="C393" t="n">
-        <v>2.255395196036164</v>
-      </c>
-    </row>
-    <row r="394">
-      <c r="A394" t="n">
-        <v>9802000384</v>
-      </c>
-      <c r="B394" t="n">
-        <v>5.989837791654287</v>
-      </c>
-      <c r="C394" t="n">
-        <v>2.178408624582164</v>
-      </c>
-    </row>
-    <row r="395">
-      <c r="A395" t="n">
-        <v>9826750464</v>
-      </c>
-      <c r="B395" t="n">
-        <v>5.936748010441494</v>
-      </c>
-      <c r="C395" t="n">
-        <v>2.256846809516075</v>
-      </c>
-    </row>
-    <row r="396">
-      <c r="A396" t="n">
-        <v>9851499520</v>
-      </c>
-      <c r="B396" t="n">
-        <v>5.924278982639498</v>
-      </c>
-      <c r="C396" t="n">
-        <v>2.309288544297972</v>
-      </c>
-    </row>
-    <row r="397">
-      <c r="A397" t="n">
-        <v>9876249600</v>
-      </c>
-      <c r="B397" t="n">
-        <v>5.862654413683829</v>
-      </c>
-      <c r="C397" t="n">
-        <v>2.21752137726327</v>
-      </c>
-    </row>
-    <row r="398">
-      <c r="A398" t="n">
-        <v>9900999680</v>
-      </c>
-      <c r="B398" t="n">
-        <v>5.864398787708184</v>
-      </c>
-      <c r="C398" t="n">
-        <v>2.274593079819441</v>
-      </c>
-    </row>
-    <row r="399">
-      <c r="A399" t="n">
-        <v>9925749760</v>
-      </c>
-      <c r="B399" t="n">
-        <v>5.876591285147287</v>
-      </c>
-      <c r="C399" t="n">
-        <v>2.320924271429033</v>
-      </c>
-    </row>
-    <row r="400">
-      <c r="A400" t="n">
-        <v>9950499840</v>
-      </c>
-      <c r="B400" t="n">
-        <v>5.860772285312891</v>
-      </c>
-      <c r="C400" t="n">
-        <v>2.271345366092218</v>
-      </c>
-    </row>
-    <row r="401">
-      <c r="A401" t="n">
-        <v>9975249920</v>
-      </c>
-      <c r="B401" t="n">
-        <v>5.812497304458483</v>
-      </c>
-      <c r="C401" t="n">
-        <v>2.362356933719642</v>
-      </c>
-    </row>
-    <row r="402">
-      <c r="A402" t="n">
-        <v>10000000000</v>
-      </c>
-      <c r="B402" t="n">
-        <v>5.817604142464508</v>
-      </c>
-      <c r="C402" t="n">
-        <v>2.329123381908004</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>